<commit_message>
ML_PL email alert created
</commit_message>
<xml_diff>
--- a/ML_PL_new/fuzz_teams.xlsx
+++ b/ML_PL_new/fuzz_teams.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="388">
   <si>
     <t>Country</t>
   </si>
@@ -1180,6 +1180,9 @@
   </si>
   <si>
     <t>PSV</t>
+  </si>
+  <si>
+    <t>Sunderland</t>
   </si>
 </sst>
 </file>
@@ -1544,7 +1547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -4965,6 +4968,9 @@
       <c r="B152" t="s">
         <v>378</v>
       </c>
+      <c r="E152" t="s">
+        <v>378</v>
+      </c>
       <c r="F152" t="s">
         <v>378</v>
       </c>
@@ -4979,11 +4985,25 @@
       <c r="B153" t="s">
         <v>380</v>
       </c>
+      <c r="E153" t="s">
+        <v>380</v>
+      </c>
       <c r="F153" t="s">
         <v>380</v>
       </c>
       <c r="G153" t="s">
         <v>381</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>7</v>
+      </c>
+      <c r="B154" t="s">
+        <v>387</v>
+      </c>
+      <c r="E154" t="s">
+        <v>387</v>
       </c>
     </row>
   </sheetData>

</xml_diff>